<commit_message>
Add Taiwan and Mexico buyer sheets to Excel
Sheet 4 - 台湾バイヤーリスト: 10 companies
  - Focus: BR380JG potential buyers and Japanese used machinery importers
  - Key targets: 鑫輝機械 (TOKU crusher dealer), 互益機械 (Japan import specialist)
  - Includes Komatsu TW distributor, Facebook-active dealers

Sheet 5 - メキシコバイヤーリスト: 8 companies
  - Focus: Used Japanese construction machinery buyers (CAT-heavy)
  - Key targets: MADISA-CAT (Mexico's largest CAT dealer),
    Ritchie Bros Mexico (84 CAT excavator imports), Maquinaria Wiebe
  - Contacts: emails, phones, Facebook, LinkedIn included

https://claude.ai/code/session_01CWtZqEG3WiurJDGDiej1wZ
</commit_message>
<xml_diff>
--- a/overseas_buyers_BR380JG3.xlsx
+++ b/overseas_buyers_BR380JG3.xlsx
@@ -10,9 +10,13 @@
     <sheet name="海外バイヤーリスト" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="プラットフォーム一覧" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="SNSアカウント一覧" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="台湾バイヤーリスト" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="メキシコバイヤーリスト" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'海外バイヤーリスト'!$A$1:$M$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'台湾バイヤーリスト'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'メキシコバイヤーリスト'!$A$1:$L$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,7 +43,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +80,16 @@
         <fgColor rgb="0092D050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00538135"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -103,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -125,6 +139,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2362,4 +2382,1172 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>優先度</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>会社名（中文）</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>会社名（日本語）</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>所在地（台湾）</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>ウェブサイト</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>メールアドレス</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>電話番号</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Facebook / SNS</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>日本製機械取扱</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>BR380JG関連</t>
+        </is>
+      </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="52" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>鑫輝機械有限公司</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>シンフェイ機械</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>基隆市七堵区</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bmcl.com.tw</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>bmcl66@mail2000.com.tw</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>02-24579141</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>◎ 日本TOKU製新品破砕機・中古建機を扱う</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>日本TOKU製新品クラッシャー（破碎機）販売実績あり</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>日本TOKUの新品クラッシャー代理店かつ中古ショベル・ブルドーザー等も扱う。BR380JG（移動式ジョークラッシャー）の需要が高い。最優先ターゲット。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="52" customHeight="1">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>互益機械有限公司（互助重機）</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>フーイー機械</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>高雄市大社区</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.huyih.com</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>huyih.hy@msa.hinet.net</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>07-3535686</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>http://huyih.blogspot.com/</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>◎ 外匯（日本）中古重機専門</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>日本からの中古ショベル輸入実績あり</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>「外匯中古重機」専門業者（外匯＝海外からの輸入）。日本製コマツ・日立・CAT等の中古ショベル・ブルドーザーを買取・販売。破砕機ニーズも高い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>台松堆高機股份有限公司</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>台松フォークリフト（Komatsu台湾代理店）</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>台北市</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>http://www.taiwan-komatsu.tw</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/taiwan.komatsu/</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>◎ コマツ台湾正規代理店</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>コマツ全製品取扱（フォークリフト中心）</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>日本小松台湾区総代理店。主にフォークリフト中心だが建設機械・コマツ全製品を取扱。BR380JG需要の把握・紹介元として重要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>鴻聖重機有限公司</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ホンセン重機</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>彰化県</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hs-digger.com.tw</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>◎ 中古ショベル・建機買取販売</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>中古建機輸入業者</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>1997年創業。工地（建設現場）・外匯（日本）からの中古ショベル・ブルドーザー等を専門に売買。日本からの輸入実績あり。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>洪鐵重機械股份有限公司</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ホンティエ重機</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>台湾（北部）</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hung-tieh.com.tw</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>◎ 日本製中古重機</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>日本製中古建機輸入・販売</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>日本製中古ショベル・ローダー・ロードローラー・発電機・堆高機（フォークリフト）等を扱う。日本からの輸入メイン。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>鉅工堆高機</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>キョコウフォークリフト</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.the-giant.com.tw</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>◎ コマツ代理権取得</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>コマツ電動フォークリフト代理</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>コマツ電動式フォークリフト代理権取得業者。コマツネットワーク活用でBR380JG導入実績業者への紹介が期待できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>台明重工</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>タイメン重工</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>http://www.backhoe.com.tw</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>◎ 中古ショベル売買</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>中古建機売買</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>中古ショベル（怪手・挖土機）専門。日本輸入品を扱う可能性あり。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>勵國重機有限公司</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>リーグオ重機</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>新北市</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Webサイト確認中</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/UsedShovelLoader/</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>◎ コマツ中古重機のFacebook投稿あり</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Komatsu WA450-3等の中古重機をFacebook上で販売</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>Facebook上でKomatsu WA450-3等の中古重機を販売。コマツファン層。BR380JGに興味を持つ可能性が高い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Hitachi Construction Machinery Taiwan</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>日立建機台湾</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>台湾（公式代理店）</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hitachicm.com.tw</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>◎ 日立建機台湾公式</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>日立製品のみ</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>日立建機の台湾公式代理店。競合だが、建設・採石業界へのネットワークを通じてBR380JGのニーズを探る情報源として活用可。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>豐悅企業有限公司</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>ホンユエ企業</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.fycmg.com</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>◎ 台湾柳工代理店・重機全般</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>建設機械全般</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>台湾柳工（LiuGong）代理店。ショベル・ローダー・プッシャー・フォークリフト・圧路機・ブルドーザー等取扱。破砕機ニーズ調査先として有望。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>優先度</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>会社名</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>所在地（メキシコ）</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>ウェブサイト</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>メールアドレス</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>電話番号</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Facebook / SNS</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>日本製機械取扱</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>CATメイン</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="52" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Maquinas Diesel S.A. de C.V. (MADISA-CAT)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Av. Industriales del Poniente 2300, Santa Catarina, Nuevo León, 66350</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://madisa.com.mx</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>+52 81 8400 2000</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>◎ CAT公認代理店</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>YES – CAT専門・メキシコ最大</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>メキシコ最大のCaterpillar正規代理店（1946年創業）。建設・鉱山・石油ガス・農業向け。Telsmith社製クラッシャーも扱う。日本製CAT中古機の輸入購買実績が期待できる最重要ターゲット。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="52" customHeight="1">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Ritchie Bros. Auctioneers de Mexico</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Polotitlan, Estado de Mexico（競売場）</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rbauction.com</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Webより確認</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>◎ 国際オークション・輸入実績多数</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>YES – CAT輸入84件</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>メキシコ向けCAT掘削機を84件輸入した実績あり（輸入統計）。メキシコ国内で定期競売を開催。日本製中古CAT建機を競売出品すれば直接リーチ可能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Maquinaria Wiebe KM 24 S.A. de C.V.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Km 24 Carretera Cuauhtémoc a Álvaro Obregón, Cuauhtémoc, Chihuahua</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.maquinariaw.com</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>awiebe71@hotmail.com
+ventas@maquinariaw.com.mx</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>+52 625 134 4523</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/maquinariaw/</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>◎ 中古CAT・建機売買専門</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>YES – CAT 320C・CAT 349FL等多数</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>メキシコ最大級の中古建機ディーラー（MachineryTraderに1,500件超の出品）。CAT掘削機・クレーン・フォークリフト等を扱う。米国・日本からの輸入品を販売。メール・Facebookで連絡可。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Tracsa S.A.P.I. de C.V. (Grupo Tracsa)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Periferico Sur 7800, Santa Maria Tequepexpan, 45600 Tlaquepaque, Jalisco</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>https://tracsa.com.mx</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Webより確認</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tracsacat</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>◎ CAT公認代理店（西部・バヒオ地方）</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>YES – CAT専門</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>メキシコ西部・バヒオ地方のCAT正規代理店（1974年〜）。14拠点。年商5億ドル超（2025年）。建設・農業・鉱業・物流。新旧CAT機械取扱。LinkedIn: Tracsa Cat。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>TMR – Tractores y Maquinaria Real</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Carretera Miguel Alemán 102 (Km 12.5), San Nicolás de los Garza, Nuevo León</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tmr.com.mx</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>+52 81 8327 0948</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tractores-y-maquinaria-real/</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>◎ CAT公認代理店（北部）</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>YES – CAT専門</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>モンテレイ・サルティーヨ・トレオン拠点のCAT公認ディーラー。新旧重機・建機の販売・レンタル。Dynapac代理店も兼任。北部メキシコ最大拠点の一つ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Empresas MATCO S.A. de C.V. (Matco Cat)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Sufragio Efectivo Norte 870, Col. Centro, Ciudad Obregón, Sonora
+他: Mexicali / Mazatlán / Culiacán / Los Mochis / Hermosillo</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>https://matco.com.mx</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>m***@matco.com.mx (ZoomInfo経由要確認)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Webより確認</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/empresas-matco-s-a-de-c-v-/</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>◎ CAT公認代理店（西部・北西部）</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>YES – CAT 300モデル以上</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>ソノラ州・バハカリフォルニア州等のCAT正規代理店。300モデル以上の機械カタログ。農業・建設・鉱業・海事。Astec Telsmith製クラッシャーも販売。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Heavy Machine México</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>メキシコ（詳細要確認）</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://heavymachine.com.mx</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Webより確認</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>◎ 中古CAT・建機全般</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>YES – CAT含む複数ブランド</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>CAT・Case・Bobcat・JD・JCB等の中古重機を扱うメキシコの建機ディーラー。日本製中古機も取扱可能性あり。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>MarketBook México</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>メキシコ全土（オンラインマーケット）</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.marketbook.mx</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Webフォームより</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>◎ 中古建機マーケットプレイス</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>YES – 各ブランド掲載</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>メキシコ国内最大級の中古農業機械・建機オンラインマーケット。出品掲載でメキシコのバイヤーに直接リーチ可能。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>